<commit_message>
Update Tendo Monitoring Data Files
- Updated multiple Excel files related to the Tendo Funnel and Model Monitoring Dashboards, reflecting the latest data as of December 25, 2023.
- Changes include:
  - New funnel data files: `20260330_New_Tendo_Funnel_sc2_0_monthlytilldec25.xlsx`, `20260330_New_Tendo_Funnel_scorecard2_0_monthlydec25.xlsx`, `20260330_New_Tendo_Funnel_scorecard2_0_peso_dec25.xlsx`, and `20260330_New_Tendo_Funnel_scorecard2_0_peso_monthly_dec25.xlsx`.
  - Updated dashboard requirements file: `20260330_Tendo_Model_Monitoring_Dashboards_Requirement_v1.pptx`.
  - Revised peso rate files: `20260330_v1pesorate.xlsx` and `20260330_v1pesorateunit.xlsx`.
  - Deleted temporary file: `~$20260330_New_Tendo_Funnel_scorecard2_0_peso_dec25.xlsx`.
</commit_message>
<xml_diff>
--- a/Tendo_Monitoring_data/20260330_New_Tendo_Funnel_sc2_0_monthlytilldec25.xlsx
+++ b/Tendo_Monitoring_data/20260330_New_Tendo_Funnel_sc2_0_monthlytilldec25.xlsx
@@ -58,22 +58,22 @@
     <t>2025-12</t>
   </si>
   <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
     <t>F</t>
   </si>
   <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>E</t>
+    <t>B</t>
   </si>
   <si>
     <t>A</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>B</t>
   </si>
 </sst>
 </file>
@@ -468,16 +468,19 @@
         <v>14</v>
       </c>
       <c r="D2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -491,19 +494,19 @@
         <v>15</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>100</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -543,19 +546,16 @@
         <v>17</v>
       </c>
       <c r="D5">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="E5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -569,19 +569,19 @@
         <v>18</v>
       </c>
       <c r="D6">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
         <v>3</v>
       </c>
-      <c r="F6">
-        <v>3</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
       <c r="H6">
-        <v>33.33</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -598,16 +598,16 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7">
         <v>5</v>
       </c>
       <c r="G7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -618,22 +618,22 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D8">
-        <v>37</v>
+        <v>289</v>
       </c>
       <c r="E8">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F8">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H8">
-        <v>66.67</v>
+        <v>73.08</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -644,22 +644,22 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D9">
-        <v>289</v>
+        <v>141</v>
       </c>
       <c r="E9">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F9">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="G9">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H9">
-        <v>69.23</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -670,22 +670,22 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D10">
-        <v>39</v>
+        <v>489</v>
       </c>
       <c r="E10">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="F10">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="G10">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="H10">
-        <v>80</v>
+        <v>85.37</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -699,19 +699,19 @@
         <v>14</v>
       </c>
       <c r="D11">
-        <v>140</v>
+        <v>39</v>
       </c>
       <c r="E11">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F11">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G11">
         <v>4</v>
       </c>
       <c r="H11">
-        <v>44.44</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -722,22 +722,22 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D12">
-        <v>489</v>
+        <v>37</v>
       </c>
       <c r="E12">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="F12">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="G12">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="H12">
-        <v>78.05</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -748,22 +748,22 @@
         <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D13">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E13">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F13">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="G13">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="H13">
-        <v>66.67</v>
+        <v>44.44</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -774,22 +774,22 @@
         <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D14">
-        <v>39</v>
+        <v>112</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>55.56</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -803,19 +803,19 @@
         <v>19</v>
       </c>
       <c r="D15">
-        <v>237</v>
+        <v>279</v>
       </c>
       <c r="E15">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F15">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G15">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="H15">
-        <v>150</v>
+        <v>51.85</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -826,22 +826,22 @@
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D16">
-        <v>112</v>
+        <v>148</v>
       </c>
       <c r="E16">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F16">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="G16">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H16">
-        <v>55.56</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -852,7 +852,7 @@
         <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D17">
         <v>48</v>
@@ -878,22 +878,22 @@
         <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D18">
-        <v>279</v>
+        <v>237</v>
       </c>
       <c r="E18">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F18">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G18">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="H18">
-        <v>51.85</v>
+        <v>150</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -904,22 +904,22 @@
         <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D19">
-        <v>148</v>
+        <v>39</v>
       </c>
       <c r="E19">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F19">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G19">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H19">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -933,19 +933,19 @@
         <v>14</v>
       </c>
       <c r="D20">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="E20">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F20">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G20">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H20">
-        <v>83.33</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -956,22 +956,22 @@
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D21">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="E21">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F21">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H21">
-        <v>33.33</v>
+        <v>83.33</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -982,22 +982,22 @@
         <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D22">
-        <v>49</v>
+        <v>227</v>
       </c>
       <c r="E22">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="F22">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="G22">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="H22">
-        <v>75</v>
+        <v>95.45</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1008,22 +1008,22 @@
         <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D23">
-        <v>227</v>
+        <v>146</v>
       </c>
       <c r="E23">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F23">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="G23">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="H23">
-        <v>90.91</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1034,22 +1034,22 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D24">
-        <v>381</v>
+        <v>29</v>
       </c>
       <c r="E24">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="F24">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="G24">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="H24">
-        <v>100</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1060,22 +1060,22 @@
         <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D25">
-        <v>146</v>
+        <v>381</v>
       </c>
       <c r="E25">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="F25">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="G25">
-        <v>3</v>
+        <v>46</v>
       </c>
       <c r="H25">
-        <v>33.33</v>
+        <v>102.22</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1086,7 +1086,7 @@
         <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D26">
         <v>137</v>
@@ -1112,19 +1112,19 @@
         <v>11</v>
       </c>
       <c r="C27" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D27">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="E27">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F27">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G27">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H27">
         <v>50</v>
@@ -1138,22 +1138,22 @@
         <v>11</v>
       </c>
       <c r="C28" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D28">
-        <v>195</v>
+        <v>49</v>
       </c>
       <c r="E28">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="F28">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="G28">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="H28">
-        <v>72.22</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1164,22 +1164,22 @@
         <v>11</v>
       </c>
       <c r="C29" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D29">
-        <v>60</v>
+        <v>107</v>
       </c>
       <c r="E29">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F29">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H29">
-        <v>50</v>
+        <v>90</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1190,22 +1190,22 @@
         <v>11</v>
       </c>
       <c r="C30" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D30">
-        <v>107</v>
+        <v>195</v>
       </c>
       <c r="E30">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F30">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="G30">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="H30">
-        <v>60</v>
+        <v>72.22</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1216,7 +1216,7 @@
         <v>11</v>
       </c>
       <c r="C31" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D31">
         <v>27</v>
@@ -1242,22 +1242,22 @@
         <v>12</v>
       </c>
       <c r="C32" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D32">
-        <v>61</v>
+        <v>100</v>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F32">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H32">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1271,19 +1271,19 @@
         <v>18</v>
       </c>
       <c r="D33">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E33">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F33">
         <v>22</v>
       </c>
       <c r="G33">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H33">
-        <v>106.67</v>
+        <v>88.23999999999999</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -1294,22 +1294,22 @@
         <v>12</v>
       </c>
       <c r="C34" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D34">
-        <v>123</v>
+        <v>61</v>
       </c>
       <c r="E34">
         <v>5</v>
       </c>
       <c r="F34">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H34">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -1320,22 +1320,22 @@
         <v>12</v>
       </c>
       <c r="C35" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D35">
-        <v>105</v>
+        <v>278</v>
       </c>
       <c r="E35">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F35">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="G35">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="H35">
-        <v>120</v>
+        <v>106.67</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -1346,22 +1346,22 @@
         <v>12</v>
       </c>
       <c r="C36" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D36">
-        <v>284</v>
+        <v>105</v>
       </c>
       <c r="E36">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="F36">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="G36">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="H36">
-        <v>88.23999999999999</v>
+        <v>120</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -1372,22 +1372,22 @@
         <v>12</v>
       </c>
       <c r="C37" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D37">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="E37">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F37">
         <v>3</v>
       </c>
       <c r="G37">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H37">
-        <v>100</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -1398,22 +1398,22 @@
         <v>13</v>
       </c>
       <c r="C38" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D38">
-        <v>80</v>
+        <v>392</v>
       </c>
       <c r="E38">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F38">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G38">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H38">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -1424,22 +1424,22 @@
         <v>13</v>
       </c>
       <c r="C39" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D39">
-        <v>149</v>
+        <v>80</v>
       </c>
       <c r="E39">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F39">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G39">
         <v>1</v>
       </c>
       <c r="H39">
-        <v>33.33</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -1450,22 +1450,22 @@
         <v>13</v>
       </c>
       <c r="C40" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D40">
-        <v>392</v>
+        <v>149</v>
       </c>
       <c r="E40">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F40">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="G40">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H40">
-        <v>88.89</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -1476,18 +1476,21 @@
         <v>13</v>
       </c>
       <c r="C41" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D41">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41">
         <v>0</v>
       </c>
-      <c r="F41">
-        <v>2</v>
-      </c>
-      <c r="G41">
+      <c r="H41">
         <v>0</v>
       </c>
     </row>
@@ -1499,7 +1502,7 @@
         <v>13</v>
       </c>
       <c r="C42" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D42">
         <v>308</v>
@@ -1528,18 +1531,15 @@
         <v>17</v>
       </c>
       <c r="D43">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G43">
-        <v>0</v>
-      </c>
-      <c r="H43">
         <v>0</v>
       </c>
     </row>

</xml_diff>